<commit_message>
update ozon ff boxes 2026-07-09
</commit_message>
<xml_diff>
--- a/supplies/117111449-1.xlsx
+++ b/supplies/117111449-1.xlsx
@@ -481,7 +481,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>В пути</t>
+          <t>ACCEPTANCE_AT_STORAGE_WAREHOUSE</t>
         </is>
       </c>
     </row>
@@ -561,7 +561,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
     </row>

</xml_diff>